<commit_message>
auto: actualización caché 2026-09-08 11:00:44
</commit_message>
<xml_diff>
--- a/CONTROL_UBI_cache.xlsx
+++ b/CONTROL_UBI_cache.xlsx
@@ -212,13 +212,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B5AE4DFC-C894-4168-94EA-659E34DF4D60}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9D4EA83-33D2-4C72-A7B3-F90EF34BFD7A}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{23DD6695-70F0-415E-B4C0-A76D51EDD25B}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7255C9FC-B894-4579-904C-EB1F8F974C34}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DA7EFCC7-8083-42BF-8511-A3EEB5317759}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{603E15E8-FC84-4866-978F-424C66B2EA70}"/>
 </file>
</xml_diff>